<commit_message>
Audit d'ergonomie : relecture appliquée aux maquettes, au rapport et aux grilles
- 20 maquettes : gabarit d'annotations commun, en-tête et pied de page de MQ-01,
  données fictives cohérentes (commande N-2026-0007, séries de la démo, photos),
  rendus refaits en page entière (bureau 1440 × 900, Pixel 7 densité 2)
- section Maquettes complétée, README des maquettes, vignettes, chemins d'images
  dans donnees-audit.json
- RGAA : plus de taux publié ; références de critères corrigées ; plan d'action
  aligné sur l'audit SEO

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit-ergonomie-2026-10-16/grilles/rgaa-site-public.xlsx
+++ b/docs/audit-ergonomie-2026-10-16/grilles/rgaa-site-public.xlsx
@@ -536,15 +536,16 @@
           <t>Taux de conformité</t>
         </is>
       </c>
-      <c r="B9" s="3">
-        <f>IF(B8&gt;0,"non calculable : "&amp;B8&amp;" critère(s) non testé(s)",IF(B5+B6=0,"—",B5/(B5+B6)))</f>
-        <v/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>non calculé : échantillon non réglementaire, restitution au lecteur d’écran non testée (7.1, 7.5)</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Le taux (C / (C + NC)) ne se calcule que lorsque plus aucun critère n'est NT : complétez la grille.</t>
+          <t>Aucun taux n'est calculé : seuls les effectifs sont donnés. Ce n'est pas une déclaration d'accessibilité.</t>
         </is>
       </c>
     </row>

</xml_diff>